<commit_message>
feat: Add CreateCustomerPage with New button workflow
</commit_message>
<xml_diff>
--- a/test-data/customer-data.xlsx
+++ b/test-data/customer-data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\RamyaBIN\totp-playwright\test-data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2FE7FB6-E292-44F9-B727-8049516121B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{735E8466-BA7B-4FCF-B34C-A6A7A55418A8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,28 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="28">
-  <si>
-    <t>First Name</t>
-  </si>
-  <si>
-    <t>Last Name Prefix</t>
-  </si>
-  <si>
-    <t>Last Name</t>
-  </si>
-  <si>
-    <t>Customer Group</t>
-  </si>
-  <si>
-    <t>Delivery Terms</t>
-  </si>
-  <si>
-    <t>Delivery Mode</t>
-  </si>
-  <si>
-    <t>ZIP Code</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="32" uniqueCount="30">
   <si>
     <t>10</t>
   </si>
@@ -104,6 +83,33 @@
   </si>
   <si>
     <t>Srinivasan</t>
+  </si>
+  <si>
+    <t>Person</t>
+  </si>
+  <si>
+    <t>Type</t>
+  </si>
+  <si>
+    <t>FirstName</t>
+  </si>
+  <si>
+    <t>LastNamePrefix</t>
+  </si>
+  <si>
+    <t>LastName</t>
+  </si>
+  <si>
+    <t>CustomerGroup</t>
+  </si>
+  <si>
+    <t>DeliveryTerms</t>
+  </si>
+  <si>
+    <t>DeliveryMode</t>
+  </si>
+  <si>
+    <t>ZIPCode</t>
   </si>
 </sst>
 </file>
@@ -480,113 +486,125 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:H4"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="13.796875" customWidth="1"/>
-    <col min="2" max="2" width="16.8984375" customWidth="1"/>
-    <col min="3" max="3" width="25.59765625" customWidth="1"/>
-    <col min="4" max="4" width="14.8984375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.296875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="13.09765625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.796875" customWidth="1"/>
+    <col min="3" max="3" width="16.8984375" customWidth="1"/>
+    <col min="4" max="4" width="9.59765625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14.8984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.296875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="13.09765625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>22</v>
+      </c>
+      <c r="B1" t="s">
+        <v>23</v>
+      </c>
+      <c r="C1" t="s">
+        <v>24</v>
+      </c>
+      <c r="D1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E1" t="s">
+        <v>26</v>
+      </c>
+      <c r="F1" t="s">
+        <v>27</v>
+      </c>
+      <c r="G1" t="s">
+        <v>28</v>
+      </c>
+      <c r="H1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" t="s">
+        <v>18</v>
+      </c>
+      <c r="C2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="F2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" t="s">
+      <c r="G2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="H2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B3" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="C3" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="D3" t="s">
         <v>6</v>
       </c>
+      <c r="E3" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" t="s">
+        <v>8</v>
+      </c>
+      <c r="G3" t="s">
+        <v>9</v>
+      </c>
+      <c r="H3" t="s">
+        <v>10</v>
+      </c>
     </row>
-    <row r="2" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" t="s">
-        <v>26</v>
-      </c>
-      <c r="C2" t="s">
-        <v>27</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B4" t="s">
         <v>11</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C4" t="s">
         <v>12</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D4" t="s">
         <v>13</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E4" t="s">
         <v>14</v>
       </c>
-      <c r="E3" t="s">
+      <c r="F4" t="s">
         <v>15</v>
       </c>
-      <c r="F3" t="s">
+      <c r="G4" t="s">
         <v>16</v>
       </c>
-      <c r="G3" t="s">
+      <c r="H4" t="s">
         <v>17</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
-        <v>18</v>
-      </c>
-      <c r="B4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
-      </c>
-      <c r="D4" t="s">
-        <v>21</v>
-      </c>
-      <c r="E4" t="s">
-        <v>22</v>
-      </c>
-      <c r="F4" t="s">
-        <v>23</v>
-      </c>
-      <c r="G4" t="s">
-        <v>24</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:G1 A3:G4 D2:G2" numberStoredAsText="1"/>
+    <ignoredError sqref="B3:H4 E2:H2" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>